<commit_message>
fixed excel format 🥶
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\images\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449CDE3E-3CDA-48A6-99FC-0348141BBDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161112AB-E90D-4142-9FCC-A173D57155C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
   <sheets>
     <sheet name="oliver" sheetId="2" r:id="rId1"/>
@@ -91,7 +91,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -424,12 +424,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
   <dimension ref="B2:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="52.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="4" max="4" width="52.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -440,7 +441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>3</v>
       </c>
@@ -459,12 +460,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
   <dimension ref="B2:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="52.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="4" max="4" width="52.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -475,7 +477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
added sequencer schematic, pin doc
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E9A8F4-0A9D-4734-9016-14B2CFB67A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3749A8-8D9B-4383-A05F-14DEC481C560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="7">
   <si>
     <t>Datum</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>proto-sequencer firmware</t>
+  </si>
+  <si>
+    <t>sequencer</t>
   </si>
 </sst>
 </file>
@@ -427,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B2:D6"/>
+  <dimension ref="B2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -487,6 +490,17 @@
       </c>
       <c r="D6" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B7" s="1">
+        <v>45894</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished io unit and frontpanel
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A053EB-104D-479F-83FC-028923C4D238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE36C4F9-E732-423F-82AB-6F1E46D2D7F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
   <si>
     <t>Datum</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>sequencer pcb</t>
+  </si>
+  <si>
+    <t>io unit schematic and pcb</t>
+  </si>
+  <si>
+    <t>frontpanel schematic and pcb</t>
   </si>
 </sst>
 </file>
@@ -433,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B2:D8"/>
+  <dimension ref="B2:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -515,6 +521,28 @@
       </c>
       <c r="D8" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B9" s="1">
+        <v>45897</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B10" s="1">
+        <v>45897</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sequencer goto hell 🥀
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE36C4F9-E732-423F-82AB-6F1E46D2D7F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6227DB57-67EF-4ABD-A492-F028E2482F9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
   <si>
     <t>Datum</t>
   </si>
@@ -57,16 +57,13 @@
     <t>proto-sequencer firmware</t>
   </si>
   <si>
-    <t>sequencer</t>
-  </si>
-  <si>
     <t>sequencer pcb</t>
   </si>
   <si>
-    <t>io unit schematic and pcb</t>
-  </si>
-  <si>
-    <t>frontpanel schematic and pcb</t>
+    <t>io unit pcb</t>
+  </si>
+  <si>
+    <t>frontpanel pcb</t>
   </si>
 </sst>
 </file>
@@ -439,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B2:D10"/>
+  <dimension ref="B2:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -506,32 +503,32 @@
         <v>45894</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B8" s="1">
-        <v>45896</v>
+        <v>45894</v>
       </c>
       <c r="C8">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
-        <v>45897</v>
+        <v>45896</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.45">
@@ -539,10 +536,32 @@
         <v>45897</v>
       </c>
       <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B11" s="1">
+        <v>45897</v>
+      </c>
+      <c r="C11">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
-        <v>9</v>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B12" s="1">
+        <v>45897</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add hours for protocol implementation
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EDEC567-84BD-4FB4-9F96-46447CA91D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C46C7D-5E10-40EE-AC1F-605122AD680D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
   <sheets>
     <sheet name="oliver" sheetId="2" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Hora</t>
   </si>
   <si>
-    <t>21.08.2025</t>
-  </si>
-  <si>
     <t>USB Treiber 💀</t>
   </si>
   <si>
@@ -67,6 +64,9 @@
   </si>
   <si>
     <t>peripherals review and order</t>
+  </si>
+  <si>
+    <t>Bridge - Protokoll</t>
   </si>
 </sst>
 </file>
@@ -107,7 +107,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -439,14 +439,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B2:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B1:D13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="4" max="4" width="52.73046875" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="4" max="4" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C1">
+        <f>SUM(C3:C10000)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -457,18 +463,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B3" t="s">
-        <v>3</v>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
+        <v>45890</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>45891</v>
       </c>
@@ -476,10 +482,10 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>45892</v>
       </c>
@@ -487,10 +493,10 @@
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>45893</v>
       </c>
@@ -498,10 +504,10 @@
         <v>0.5</v>
       </c>
       <c r="D6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>45894</v>
       </c>
@@ -509,10 +515,10 @@
         <v>0.5</v>
       </c>
       <c r="D7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>45894</v>
       </c>
@@ -520,10 +526,10 @@
         <v>0.5</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>45896</v>
       </c>
@@ -531,10 +537,10 @@
         <v>1.5</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>45897</v>
       </c>
@@ -542,10 +548,10 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.45">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>45897</v>
       </c>
@@ -553,10 +559,10 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>45897</v>
       </c>
@@ -564,10 +570,10 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <v>45898</v>
       </c>
@@ -575,7 +581,7 @@
         <v>0.5</v>
       </c>
       <c r="D13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -585,14 +591,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
-  <dimension ref="B2:D3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B1:D5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="4" max="4" width="52.73046875" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C1">
+        <f>SUM(C3:C10000)</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -603,15 +615,37 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B3" t="s">
-        <v>3</v>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="1">
+        <v>45890</v>
       </c>
       <c r="C3">
         <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="1">
+        <v>45892</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="1">
+        <v>45898</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated first test times
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A43432-4724-4A51-989D-CE775EFA8BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7EE8D8B-9E3D-44BC-A370-2F9638934634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
   <si>
     <t>Datum</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>assembly ax08 lite</t>
+  </si>
+  <si>
+    <t>first ax08 lite tests</t>
   </si>
 </sst>
 </file>
@@ -445,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:D15"/>
+  <dimension ref="B1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -455,7 +458,7 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>18.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.45">
@@ -610,6 +613,17 @@
       </c>
       <c r="D15" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B16" s="1">
+        <v>45901</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
first tests, added silicon errate 🥶
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026A8B9B-C9DA-4B0F-867B-3B83D1971679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BC8AEE-107A-4C33-98BC-8B0E9487E56D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="16">
   <si>
     <t>Datum</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>architecture design discussion</t>
+  </si>
+  <si>
+    <t>ax08 lite tests</t>
   </si>
 </sst>
 </file>
@@ -454,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:D19"/>
+  <dimension ref="B1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -464,7 +467,7 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.45">
@@ -663,6 +666,17 @@
       </c>
       <c r="D19" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B20" s="1">
+        <v>45903</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -672,7 +686,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
-  <dimension ref="B1:D6"/>
+  <dimension ref="B1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="11.3984375" customWidth="1"/>
@@ -682,7 +696,7 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.45">
@@ -738,6 +752,17 @@
       </c>
       <c r="D6" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B7" s="1">
+        <v>45903</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
⌛Optimize memory unit & sequencer
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66139D89-3F12-49F0-9FEE-BACBE4FFFC1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74E8052-3336-4BB4-8DB5-AEFD1C69059E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
   <si>
     <t>Datum</t>
   </si>
@@ -91,6 +91,12 @@
   </si>
   <si>
     <t>Sequencer Breadboard</t>
+  </si>
+  <si>
+    <t>Optimize &amp; test memory unit, s2p and p2s modules</t>
+  </si>
+  <si>
+    <t>Rewrite sequencer</t>
   </si>
 </sst>
 </file>
@@ -714,7 +720,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
-  <dimension ref="B1:D10"/>
+  <dimension ref="B1:D12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" customWidth="1"/>
@@ -724,7 +730,7 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>22.5</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
@@ -824,6 +830,28 @@
       </c>
       <c r="D10" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="1">
+        <v>45906</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>45906</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
⌛ Memory unit testing
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74E8052-3336-4BB4-8DB5-AEFD1C69059E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD16F0D6-367B-477D-8980-0C535FEC565D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>Datum</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>Rewrite sequencer</t>
+  </si>
+  <si>
+    <t>Testing mem unit firmware on pcb and fixing bugs</t>
   </si>
 </sst>
 </file>
@@ -720,7 +723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
-  <dimension ref="B1:D12"/>
+  <dimension ref="B1:D13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" customWidth="1"/>
@@ -730,7 +733,7 @@
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
@@ -852,6 +855,17 @@
       </c>
       <c r="D12" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <v>45907</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
⌛time update - ax08 main production
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D59567-4EC6-41FE-B3BB-E618D0BF510F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007459AA-68A8-47E6-8C17-03EE3EF93E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="84">
   <si>
     <t>Datum</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Case - Cable Anchor</t>
+  </si>
+  <si>
+    <t>assembly ax08 main</t>
   </si>
 </sst>
 </file>
@@ -664,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:E52"/>
+  <dimension ref="B1:E53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -675,7 +678,7 @@
     <row r="1" spans="2:5" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.45">
@@ -1390,6 +1393,20 @@
       </c>
       <c r="E52" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B53" s="1">
+        <v>46304</v>
+      </c>
+      <c r="C53">
+        <v>3</v>
+      </c>
+      <c r="D53" t="s">
+        <v>83</v>
+      </c>
+      <c r="E53" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
⌛ time update - ax08 integration
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007459AA-68A8-47E6-8C17-03EE3EF93E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB286AF1-2606-4F94-A3EF-C2E0D3E4EF3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="86">
   <si>
     <t>Datum</t>
   </si>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t>assembly ax08 main</t>
+  </si>
+  <si>
+    <t>assembly ax08</t>
+  </si>
+  <si>
+    <t>ax08 integration test</t>
   </si>
 </sst>
 </file>
@@ -667,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:E53"/>
+  <dimension ref="B1:E55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -678,7 +684,7 @@
     <row r="1" spans="2:5" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.45">
@@ -1407,6 +1413,34 @@
       </c>
       <c r="E53" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B54" s="1">
+        <v>46308</v>
+      </c>
+      <c r="C54">
+        <v>9</v>
+      </c>
+      <c r="D54" t="s">
+        <v>84</v>
+      </c>
+      <c r="E54" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B55" s="1">
+        <v>46308</v>
+      </c>
+      <c r="C55">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>85</v>
+      </c>
+      <c r="E55" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
⌛ time update - cables
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\project_mismanagement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89D5922-76B5-4A1D-BE04-1EB899EEF61F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A3D976-F361-4DF2-89D1-8621D8408AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
   <sheets>
     <sheet name="oliver" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="89">
   <si>
     <t>Datum</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Cutting the case lid glass of case #2</t>
+  </si>
+  <si>
+    <t>ax08 cables</t>
   </si>
 </sst>
 </file>
@@ -347,7 +350,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -363,7 +366,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -679,21 +682,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:E55"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:E56"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="4" max="4" width="52.7109375" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="52.73046875" customWidth="1"/>
+    <col min="5" max="5" width="13.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:5" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -707,7 +710,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B3" s="1">
         <v>45890</v>
       </c>
@@ -721,7 +724,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B4" s="1">
         <v>45891</v>
       </c>
@@ -735,7 +738,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B5" s="1">
         <v>45892</v>
       </c>
@@ -749,7 +752,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B6" s="1">
         <v>45893</v>
       </c>
@@ -763,7 +766,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B7" s="1">
         <v>45894</v>
       </c>
@@ -777,7 +780,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B8" s="1">
         <v>45894</v>
       </c>
@@ -791,7 +794,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>45896</v>
       </c>
@@ -805,7 +808,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" s="1">
         <v>45897</v>
       </c>
@@ -819,7 +822,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" s="1">
         <v>45897</v>
       </c>
@@ -833,7 +836,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B12" s="1">
         <v>45897</v>
       </c>
@@ -847,7 +850,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B13" s="1">
         <v>45898</v>
       </c>
@@ -861,7 +864,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B14" s="1">
         <v>45901</v>
       </c>
@@ -875,7 +878,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B15" s="1">
         <v>45901</v>
       </c>
@@ -889,7 +892,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B16" s="1">
         <v>45901</v>
       </c>
@@ -903,7 +906,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B17" s="1">
         <v>45902</v>
       </c>
@@ -917,7 +920,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B18" s="1">
         <v>45902</v>
       </c>
@@ -931,7 +934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B19" s="1">
         <v>45902</v>
       </c>
@@ -945,7 +948,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B20" s="1">
         <v>45903</v>
       </c>
@@ -959,7 +962,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B21" s="1">
         <v>45904</v>
       </c>
@@ -973,7 +976,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B22" s="1">
         <v>45904</v>
       </c>
@@ -987,7 +990,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B23" s="1">
         <v>45907</v>
       </c>
@@ -1001,7 +1004,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B24" s="1">
         <v>45909</v>
       </c>
@@ -1015,7 +1018,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B25" s="1">
         <v>45910</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B26" s="1">
         <v>45910</v>
       </c>
@@ -1043,7 +1046,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B27" s="1">
         <v>45911</v>
       </c>
@@ -1057,7 +1060,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B28" s="1">
         <v>45911</v>
       </c>
@@ -1071,7 +1074,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B29" s="1">
         <v>45912</v>
       </c>
@@ -1085,7 +1088,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B30" s="1">
         <v>45915</v>
       </c>
@@ -1099,7 +1102,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B31" s="1">
         <v>45916</v>
       </c>
@@ -1113,7 +1116,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B32" s="1">
         <v>45917</v>
       </c>
@@ -1127,7 +1130,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B33" s="1">
         <v>45917</v>
       </c>
@@ -1141,7 +1144,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B34" s="1">
         <v>45918</v>
       </c>
@@ -1155,7 +1158,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B35" s="1">
         <v>45918</v>
       </c>
@@ -1169,7 +1172,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B36" s="1">
         <v>45918</v>
       </c>
@@ -1183,7 +1186,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B37" s="1">
         <v>45919</v>
       </c>
@@ -1197,7 +1200,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B38" s="1">
         <v>45921</v>
       </c>
@@ -1211,7 +1214,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B39" s="1">
         <v>45922</v>
       </c>
@@ -1225,7 +1228,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B40" s="1">
         <v>45923</v>
       </c>
@@ -1239,7 +1242,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" s="1">
         <v>45923</v>
       </c>
@@ -1253,7 +1256,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" s="1">
         <v>45924</v>
       </c>
@@ -1267,7 +1270,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" s="1">
         <v>45924</v>
       </c>
@@ -1281,7 +1284,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" s="1">
         <v>45925</v>
       </c>
@@ -1295,7 +1298,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" s="1">
         <v>45925</v>
       </c>
@@ -1309,7 +1312,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" s="1">
         <v>46291</v>
       </c>
@@ -1323,7 +1326,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" s="1">
         <v>46291</v>
       </c>
@@ -1337,7 +1340,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" s="1">
         <v>46291</v>
       </c>
@@ -1351,7 +1354,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" s="1">
         <v>46292</v>
       </c>
@@ -1365,7 +1368,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" s="1">
         <v>46292</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" s="1">
         <v>46299</v>
       </c>
@@ -1393,7 +1396,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B52" s="1">
         <v>46300</v>
       </c>
@@ -1407,7 +1410,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B53" s="1">
         <v>46304</v>
       </c>
@@ -1421,7 +1424,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B54" s="1">
         <v>46308</v>
       </c>
@@ -1435,7 +1438,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B55" s="1">
         <v>46308</v>
       </c>
@@ -1447,6 +1450,20 @@
       </c>
       <c r="E55" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B56" s="1">
+        <v>46309</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
+      </c>
+      <c r="D56" t="s">
+        <v>88</v>
+      </c>
+      <c r="E56" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1457,20 +1474,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED3E0BF-F2BE-451D-97DA-7705BD8F1DBF}">
   <dimension ref="B1:F51"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="52.7109375" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" customWidth="1"/>
+    <col min="4" max="4" width="52.73046875" customWidth="1"/>
+    <col min="5" max="5" width="13.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:5" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1484,7 +1501,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B3" s="1">
         <v>45890</v>
       </c>
@@ -1498,7 +1515,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B4" s="1">
         <v>45892</v>
       </c>
@@ -1512,7 +1529,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B5" s="1">
         <v>45898</v>
       </c>
@@ -1526,7 +1543,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B6" s="1">
         <v>45902</v>
       </c>
@@ -1540,7 +1557,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B7" s="1">
         <v>45903</v>
       </c>
@@ -1554,7 +1571,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B8" s="1">
         <v>45904</v>
       </c>
@@ -1568,7 +1585,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>45904</v>
       </c>
@@ -1582,7 +1599,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" s="1">
         <v>45905</v>
       </c>
@@ -1596,7 +1613,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" s="1">
         <v>45906</v>
       </c>
@@ -1610,7 +1627,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B12" s="1">
         <v>45906</v>
       </c>
@@ -1624,7 +1641,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B13" s="1">
         <v>45907</v>
       </c>
@@ -1638,7 +1655,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B14" s="1">
         <v>45907</v>
       </c>
@@ -1652,7 +1669,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B15" s="1">
         <v>45908</v>
       </c>
@@ -1666,7 +1683,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B16" s="1">
         <v>45909</v>
       </c>
@@ -1680,7 +1697,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B17" s="1">
         <v>45910</v>
       </c>
@@ -1694,7 +1711,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B18" s="1">
         <v>45910</v>
       </c>
@@ -1708,7 +1725,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B19" s="1">
         <v>45911</v>
       </c>
@@ -1722,7 +1739,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B20" s="1">
         <v>45911</v>
       </c>
@@ -1736,7 +1753,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B21" s="1">
         <v>45912</v>
       </c>
@@ -1750,7 +1767,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B22" s="1">
         <v>45912</v>
       </c>
@@ -1764,7 +1781,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B23" s="1">
         <v>45912</v>
       </c>
@@ -1778,7 +1795,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B24" s="1">
         <v>45548</v>
       </c>
@@ -1792,7 +1809,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B25" s="1">
         <v>45915</v>
       </c>
@@ -1806,7 +1823,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B26" s="1">
         <v>45916</v>
       </c>
@@ -1823,7 +1840,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B27" s="1">
         <v>45917</v>
       </c>
@@ -1840,7 +1857,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B28" s="1">
         <v>45918</v>
       </c>
@@ -1857,7 +1874,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B29" s="1">
         <v>45919</v>
       </c>
@@ -1874,7 +1891,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B30" s="1">
         <v>45920</v>
       </c>
@@ -1891,7 +1908,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B31" s="1">
         <v>45921</v>
       </c>
@@ -1908,7 +1925,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B32" s="1">
         <v>45921</v>
       </c>
@@ -1922,7 +1939,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B33" s="1">
         <v>45922</v>
       </c>
@@ -1936,7 +1953,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B34" s="1">
         <v>45922</v>
       </c>
@@ -1950,7 +1967,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B35" s="1">
         <v>45923</v>
       </c>
@@ -1964,7 +1981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B36" s="1">
         <v>45923</v>
       </c>
@@ -1978,7 +1995,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B37" s="1">
         <v>45924</v>
       </c>
@@ -1992,7 +2009,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B38" s="1">
         <v>45924</v>
       </c>
@@ -2006,7 +2023,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B39" s="1">
         <v>45925</v>
       </c>
@@ -2020,7 +2037,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B40" s="1">
         <v>45925</v>
       </c>
@@ -2034,7 +2051,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" s="1">
         <v>45926</v>
       </c>
@@ -2048,7 +2065,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" s="1">
         <v>45926</v>
       </c>
@@ -2062,7 +2079,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" s="1">
         <v>45926</v>
       </c>
@@ -2076,7 +2093,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" s="1">
         <v>45927</v>
       </c>
@@ -2090,7 +2107,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" s="1">
         <v>45927</v>
       </c>
@@ -2104,7 +2121,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" s="1">
         <v>45928</v>
       </c>
@@ -2118,7 +2135,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" s="1">
         <v>45933</v>
       </c>
@@ -2132,7 +2149,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" s="1">
         <v>45934</v>
       </c>
@@ -2146,7 +2163,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" s="1">
         <v>45935</v>
       </c>
@@ -2160,7 +2177,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" s="1">
         <v>45944</v>
       </c>
@@ -2174,7 +2191,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" s="1">
         <v>45944</v>
       </c>

</xml_diff>

<commit_message>
⌛ time update - peripherals assembly
</commit_message>
<xml_diff>
--- a/project_mismanagement/zeiten.xlsx
+++ b/project_mismanagement/zeiten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\project_mismanagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5918ABCE-E194-423E-B45C-A73AFA64D9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6797832E-185B-49D9-985D-1111D14F7FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{8B2EF68E-96B7-4F72-8440-4EEFFDE0E6ED}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="97">
   <si>
     <t>Datum</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t>IO unit TX buffer</t>
+  </si>
+  <si>
+    <t>assembly ax08 peripherals</t>
   </si>
 </sst>
 </file>
@@ -703,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8605FC15-F497-4A19-9DC6-DDBAF4F9624E}">
-  <dimension ref="B1:E58"/>
+  <dimension ref="B1:E59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -714,7 +717,7 @@
     <row r="1" spans="2:5" x14ac:dyDescent="0.45">
       <c r="C1">
         <f>SUM(C3:C10000)</f>
-        <v>131</v>
+        <v>133.5</v>
       </c>
     </row>
     <row r="2" spans="2:5" x14ac:dyDescent="0.45">
@@ -1489,7 +1492,7 @@
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B57" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -1503,7 +1506,7 @@
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B58" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -1513,6 +1516,20 @@
       </c>
       <c r="E58" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B59" s="1">
+        <v>46312</v>
+      </c>
+      <c r="C59">
+        <v>2.5</v>
+      </c>
+      <c r="D59" t="s">
+        <v>96</v>
+      </c>
+      <c r="E59" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -2312,7 +2329,7 @@
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B56" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -2326,7 +2343,7 @@
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B57" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C57">
         <v>1</v>

</xml_diff>